<commit_message>
lign CyFun 2023/2025 with CCB sources, scoring set by framework
- Libraries match the CCB booklets and tools: EN/FR/NL texts, management aspects (IG/EG), the CCB mapping; CyFun 2025 v9, CyFun 2023 v8 regenerated from its Excel source
- New framework properties score_scale_locked and score_calculation_method (migration 0192) replace hardcoded URNs; both libraries show scores by default
- New CyFun audits: average of averages, N/A counted at the level's target, scores rounded in the backend, missing documentation score at the scale minimum
- Export picks the tool of the audit's level; CyFun 2023 can be exported; export options listed through a generic framework_exports field
- Radar chart uses get_scores_for; scoring cleanups; docs updated
</commit_message>
<xml_diff>
--- a/tools/excel/ccb/ccb-cff-2023-03-01.xlsx
+++ b/tools/excel/ccb/ccb-cff-2023-03-01.xlsx
@@ -602,10 +602,8 @@
           <t>version</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
+      <c r="B3" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="4">
@@ -767,7 +765,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -935,6 +933,42 @@
       <c r="B14" t="inlineStr">
         <is>
           <t>implementation_groups</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>score_calculation_method</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>average_of_averages</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>score_scale_locked</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>field_visibility</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>{"score": {"auditor": "edit", "respondent": "edit"}, "is_scored": {"auditor": "edit", "respondent": "edit"}, "documentation_score": {"auditor": "edit", "respondent": "edit"}}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add score defaults to minimum option
</commit_message>
<xml_diff>
--- a/tools/excel/ccb/ccb-cff-2023-03-01.xlsx
+++ b/tools/excel/ccb/ccb-cff-2023-03-01.xlsx
@@ -765,7 +765,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -969,6 +969,18 @@
       <c r="B17" t="inlineStr">
         <is>
           <t>{"score": {"auditor": "edit", "respondent": "edit"}, "is_scored": {"auditor": "edit", "respondent": "edit"}, "documentation_score": {"auditor": "edit", "respondent": "edit"}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>score_defaults_to_minimum</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>x</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
remove useless score_defaults_to_minimum flag
</commit_message>
<xml_diff>
--- a/tools/excel/ccb/ccb-cff-2023-03-01.xlsx
+++ b/tools/excel/ccb/ccb-cff-2023-03-01.xlsx
@@ -767,7 +767,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -971,18 +971,6 @@
       <c r="B17" t="inlineStr">
         <is>
           <t>{"score": {"auditor": "edit", "respondent": "edit"}, "is_scored": {"auditor": "edit", "respondent": "edit"}, "documentation_score": {"auditor": "edit", "respondent": "edit"}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>score_defaults_to_minimum</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>x</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: multiple improvements to better manage cyfun frameworks
</commit_message>
<xml_diff>
--- a/tools/excel/ccb/ccb-cff-2023-03-01.xlsx
+++ b/tools/excel/ccb/ccb-cff-2023-03-01.xlsx
@@ -602,10 +602,8 @@
           <t>version</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
+      <c r="B3" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="4">
@@ -614,8 +612,10 @@
           <t>publication_date</t>
         </is>
       </c>
-      <c r="B4" s="30" t="n">
-        <v>46255</v>
+      <c r="B4" s="30" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -767,7 +767,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -935,6 +935,42 @@
       <c r="B14" t="inlineStr">
         <is>
           <t>implementation_groups</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>score_calculation_method</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>average_of_averages</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>score_scale_locked</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>field_visibility</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>{"score": {"auditor": "edit", "respondent": "edit"}, "is_scored": {"auditor": "edit", "respondent": "edit"}, "documentation_score": {"auditor": "edit", "respondent": "edit"}}</t>
         </is>
       </c>
     </row>

</xml_diff>